<commit_message>
Initial commit dashboard streamlit
</commit_message>
<xml_diff>
--- a/dashboard/raw.xlsx
+++ b/dashboard/raw.xlsx
@@ -526,32 +526,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADD/HC/004/2027</t>
+          <t>ADD/HC/008/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30 00:00:00</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2027-09-29 00:00:00</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2087753188</t>
+          <t>2685276182</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>75318</t>
+          <t>27618</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Intan Permata</t>
+          <t>Andi Pratama</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -561,32 +561,32 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19000000</t>
+          <t>35000000</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>19000000</t>
+          <t>17500000</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Terlaksana</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Belum direalisasikan</t>
+          <t>Berhasil</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -596,27 +596,27 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>38000000</t>
+          <t>70000000</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Sudah</t>
+          <t>Terlaksana</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:00</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>THR telah direalisasikan</t>
+          <t>done yac</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Islam</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -624,37 +624,41 @@
           <t>Aktif</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>12 Bulan (349 Hari)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADD/HC/008/2026</t>
+          <t>ADD/HC/003/2027</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-11 00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2027-03-26</t>
+          <t>2027-08-10 00:00:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2685276182</t>
+          <t>2196285353</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>27618</t>
+          <t>28535</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Andi Pratama</t>
+          <t>Hendra Wijaya</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -664,32 +668,32 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>35000000</t>
+          <t>25000000</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>17500000</t>
+          <t>25000000</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Belum/Gagal</t>
+          <t>Sudah</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-12 00:00:00</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UPCT telah direalisasikan</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -699,17 +703,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>70000000</t>
+          <t>50000000</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Belum/Gagal</t>
+          <t>Terlaksana</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -719,7 +723,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Islam</t>
+          <t>-</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -727,51 +731,47 @@
           <t>Aktif</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>7 Bulan (199 Hari)</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADD/HC/003/2027</t>
+          <t>ADD/HC/002/2027</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-11 00:00:00</t>
+          <t>2026-07-25 00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2027-08-10 00:00:00</t>
+          <t>2027-07-24 00:00:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2196285353</t>
+          <t>2293764646</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>28535</t>
+          <t>76464</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Hendra Wijaya</t>
+          <t>Gina Maharani</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ProHire</t>
+          <t>ReHire</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25000000</t>
+          <t>17000000</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25000000</t>
+          <t>17000000</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-08-12 00:00:00</t>
+          <t>2026-07-25 00:00:00</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -806,22 +806,22 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>50000000</t>
+          <t>34000000</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-07-30 00:00:00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Belum direalisasikan</t>
+          <t>THR telah direalisasikan</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -839,42 +839,42 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADD/HC/002/2027</t>
+          <t>ADD/HC/001/2027</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-25 00:00:00</t>
+          <t>2026-06-17 00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2027-07-24 00:00:00</t>
+          <t>2027-06-16 00:00:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2293764646</t>
+          <t>1985312917</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>76464</t>
+          <t>31291</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Gina Maharani</t>
+          <t>Fajar Ramadhan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ReHire</t>
+          <t>ProHire</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>17000000</t>
+          <t>22000000</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>17000000</t>
+          <t>22000000</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-07-25 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -909,22 +909,22 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>34000000</t>
+          <t>44000000</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Sudah</t>
+          <t>Belum</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-07-30 00:00:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>THR telah direalisasikan</t>
+          <t>Menunggu proses realisasi</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -942,52 +942,52 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADD/HC/001/2027</t>
+          <t>ADD/HC/005/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-17 00:00:00</t>
+          <t>2026-05-08 00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2027-06-16 00:00:00</t>
+          <t>2027-05-07 00:00:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1985312917</t>
+          <t>2490904561</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>31291</t>
+          <t>90456</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Fajar Ramadhan</t>
+          <t>Eka Putri</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ProHire</t>
+          <t>ReHire</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22000000</t>
+          <t>16000000</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>22000000</t>
+          <t>8000000</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-06-18 00:00:00</t>
+          <t>2026-05-08 00:00:00</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1012,22 +1012,22 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>44000000</t>
+          <t>32000000</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-05-12 00:00:00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Menunggu proses realisasi</t>
+          <t>THR telah direalisasikan</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Selesai Kontrak / Tidak Aktif</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1045,32 +1045,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADD/HC/005/2026</t>
+          <t>ADD/HC/004/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-08 00:00:00</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-05-07 00:00:00</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2490904561</t>
+          <t>2092921785</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>90456</t>
+          <t>92178</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Eka Putri</t>
+          <t>Dimas Saputra</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1078,59 +1078,49 @@
           <t>ReHire</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>16000000</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>8000000</t>
-        </is>
+      <c r="H7" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>18000000</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Sudah</t>
+          <t>Belum</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-05-08 00:00:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>UPCT telah direalisasikan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>32000000</t>
-        </is>
+          <t>Belum direalisasikan</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>36000000</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Sudah</t>
+          <t>On Progress</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-12 00:00:00</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>THR telah direalisasikan</t>
+          <t>Menunggu acc</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1140,75 +1130,79 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Selesai Kontrak / Tidak Aktif</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>Aktif</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>12 Bulan (354 Hari)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADD/HC/004/2026</t>
+          <t>ADD/HC/003/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-04-21 00:00:00</t>
+          <t>2026-03-12 00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2027-04-20 00:00:00</t>
+          <t>2027-03-11 00:00:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2092921785</t>
+          <t>2395956432</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>92178</t>
+          <t>95643</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Dimas Saputra</t>
+          <t>Citra Lestari</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ProHire</t>
+          <t>ReHire</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>18000000</t>
+          <t>15000000</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>18000000</t>
+          <t>7500000</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-03-10 00:00:00</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Belum direalisasikan</t>
+          <t>UPCT telah direalisasikan</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1218,22 +1212,22 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>36000000</t>
+          <t>30000000</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>On Progress</t>
+          <t>Sudah</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-03-15 00:00:00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Menunggu acc</t>
+          <t>THR telah direalisasikan</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1251,87 +1245,87 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADD/HC/003/2026</t>
+          <t>ADD/HC/002/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-03-12 00:00:00</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-03-11 00:00:00</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2395956432</t>
+          <t>2288852144</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>95643</t>
+          <t>85214</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Citra Lestari</t>
+          <t>Bunga Aulia</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ReHire</t>
+          <t>ProHire</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>15000000</t>
+          <t>20000000</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>7500000</t>
+          <t>20000000</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>Terlaksana</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>UPCT telah direalisasikan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>40000000</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Sudah</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>UPCT telah direalisasikan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>30000000</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Sudah</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-03-15 00:00:00</t>
+          <t>2026-02-20 00:00:00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1341,7 +1335,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1349,57 +1343,61 @@
           <t>Aktif</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>12 Bulan (360 Hari)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADD/HC/002/2026</t>
+          <t>ADD/HC/010/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-02-03 00:00:00</t>
+          <t>2027-07-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-02-02 00:00:00</t>
+          <t>2028-05-05</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2288852144</t>
+          <t>2790837461</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>85214</t>
+          <t>83746</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bunga Aulia</t>
+          <t>Eka Putri</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ProHire</t>
+          <t>ReHire</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>20000000</t>
+          <t>25000000</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>20000000</t>
+          <t>12500000</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1409,12 +1407,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>UPCT telah direalisasikan</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1424,27 +1422,27 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>40000000</t>
+          <t>50000000</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Sudah</t>
+          <t>Belum/Gagal</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-02-20 00:00:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>THR telah direalisasikan</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Islam</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1452,52 +1450,62 @@
           <t>Aktif</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>10 Bulan (309 Hari)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADD/HC/010/2026</t>
+          <t>ADD/HC/004/2027</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027-07-01</t>
+          <t>2025-10-07</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2028-05-05</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2790837461</t>
+          <t>2087753188</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>83746</t>
+          <t>75318</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Eka Putri</t>
+          <t>Intan Permata</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ReHire</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J11" t="n">
-        <v>12500000</v>
+          <t>ProHire</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>19000000</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>19000000</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1514,11 +1522,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="N11" t="n">
-        <v>2</v>
-      </c>
-      <c r="O11" t="n">
-        <v>50000000</v>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>38000000</t>
+        </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1537,7 +1549,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Islam</t>
+          <t>-</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1547,7 +1559,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>10 Bulan (309 Hari)</t>
+          <t>12 Bulan (350 Hari)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix kalkulasi masa kontrak otomatis dan perbaiki perpanjangan SK
</commit_message>
<xml_diff>
--- a/dashboard/raw.xlsx
+++ b/dashboard/raw.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,7 +541,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2685276182</t>
+          <t>2585276182</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Selesai Kontrak / Tidak Aktif</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025-10-06</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hindu</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>12 Bulan (354 Hari)</t>
+          <t>10 Bulan (298 Hari)</t>
         </is>
       </c>
     </row>
@@ -1560,6 +1560,113 @@
       <c r="U11" t="inlineStr">
         <is>
           <t>12 Bulan (350 Hari)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ADD/HC/013/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2027-07-30</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2685923462</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>92346</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Andi Pratama</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ProHire</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>40000000</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>40000000</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Belum/Gagal</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>80000000</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Belum/Gagal</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Islam</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Aktif</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>11 Bulan (333 Hari)</t>
         </is>
       </c>
     </row>

</xml_diff>